<commit_message>
fix: facturación exitosa, falta reflejarlo en el pdf
</commit_message>
<xml_diff>
--- a/input/Facturacion.xlsx
+++ b/input/Facturacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programación\trabajo\Facturación Electronica Python\InvoicerPRO-Development\input\Factura B\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\learr\Documents\Fys\invoice-pro\invoice-pro-back\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5FEC06-1CB3-49EC-B96D-C8F84E92CB02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6021D6DF-19A4-4FC5-96D7-AFE0F3148276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-40" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Factura B" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="64">
   <si>
     <t>Fecha</t>
   </si>
@@ -234,12 +234,6 @@
   </si>
   <si>
     <t>CI Extranjera</t>
-  </si>
-  <si>
-    <t>203020</t>
-  </si>
-  <si>
-    <t>203020.00</t>
   </si>
   <si>
     <t>11</t>
@@ -860,7 +854,7 @@
         <v>32</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>33</v>
@@ -878,16 +872,16 @@
         <v>20450015262</v>
       </c>
       <c r="J2" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>37</v>
       </c>
       <c r="L2" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M2" s="7">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="N2" t="s">
         <v>38</v>
@@ -970,16 +964,16 @@
         <v>20450015262</v>
       </c>
       <c r="J3" s="7">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>37</v>
       </c>
       <c r="L3" s="7">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="M3" s="7">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="N3" t="s">
         <v>38</v>
@@ -1053,16 +1047,16 @@
         <v>20450015262</v>
       </c>
       <c r="J4" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>37</v>
       </c>
       <c r="L4" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M4" s="7">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="N4" t="s">
         <v>38</v>
@@ -1147,29 +1141,29 @@
       <c r="K5" t="s">
         <v>58</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" t="s">
+        <v>58</v>
+      </c>
+      <c r="P5" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>58</v>
+      </c>
+      <c r="R5" t="s">
+        <v>58</v>
+      </c>
+      <c r="S5" t="s">
         <v>61</v>
-      </c>
-      <c r="M5" t="s">
-        <v>62</v>
-      </c>
-      <c r="N5" t="s">
-        <v>58</v>
-      </c>
-      <c r="O5" t="s">
-        <v>58</v>
-      </c>
-      <c r="P5" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>58</v>
-      </c>
-      <c r="R5" t="s">
-        <v>58</v>
-      </c>
-      <c r="S5" t="s">
-        <v>63</v>
       </c>
       <c r="T5" t="s">
         <v>58</v>
@@ -1202,7 +1196,7 @@
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="AD6"/>
       <c r="AE6"/>

</xml_diff>